<commit_message>
Record V0 world, farm, mine and fishing decisions
</commit_message>
<xml_diff>
--- a/docs/current/LITTLE-VALLEY-CARD-REGISTER-V0.xlsx
+++ b/docs/current/LITTLE-VALLEY-CARD-REGISTER-V0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lá bài V0" sheetId="1" r:id="R903c3936c05c4bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lá bài V0" sheetId="1" r:id="R32ef8b336b3949e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -47,6 +47,15 @@
       <x:color rgb="FF1E3A5F"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -67,7 +76,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -97,6 +106,20 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -105,8 +128,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CardsV0" displayName="CardsV0" ref="A6:K34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:K34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CardsV0" displayName="CardsV0" ref="A6:K41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:K41"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Identity / tên làm việc"/>
     <x:tableColumn id="2" name="Loại lá"/>
@@ -352,7 +375,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Mỗi dòng là một identity hoặc một identity đang cần phân ranh. Tên có ghi “fixture/chưa đặt tên” chưa phải tên hiển thị cuối.</x:v>
+        <x:v>Mỗi dòng là một identity hoặc một state cần phân biệt. Tilled Soil là state của Soil, không có entry Bách Khoa riêng.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -436,16 +459,16 @@
         <x:v>World</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
-        <x:v>Bao gồm các Area</x:v>
+        <x:v>Lá gốc; chứa các Region</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>Khi World được trình bày cho người chơi</x:v>
+        <x:v>Lá duy nhất ở màn đầu</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>Mặc định không kích hoạt</x:v>
+        <x:v>Chơi World để mở tableau các lá Region</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>Không có commit trực tiếp đã chốt</x:v>
+        <x:v>Mở lá con 0 AP navigation; không tự commit action của Region</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
         <x:v>Không áp dụng</x:v>
@@ -457,49 +480,45 @@
         <x:v>Owner chốt grammar</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>Cách trình bày World chưa chốt; không ép lá
-vuông trên tableau</x:v>
+        <x:v>Danh sách Region V0 và nhãn loại Region/Area còn cần đồng bộ</x:v>
       </x:c>
       <x:c r="K7" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-00, UI-27, UI-37</x:v>
+        <x:v>Decision 09 · CG-35/37, UI-37; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" s="10" t="str">
-        <x:v>Home / Farm (nhãn fixture)</x:v>
+        <x:v>Home</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Area</x:v>
+        <x:v>Region card</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Thuộc World</x:v>
+        <x:v>Lá con của World</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Area Home/Farm được người chơi nhìn thấy</x:v>
+        <x:v>Khi chơi World và lá Home hiện trên tableau Region</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Chứa plot, Farmhouse và Shipping Bin trong
-fixture</x:v>
+        <x:v>Chạm Home mở tableau chứa Field, Farmhouse, Shipping Bin</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Area giữ state khi cuộn đi; bản thân Area
-không là target bắt buộc</x:v>
+        <x:v>Mở Home 0 AP navigation; lá con giữ state riêng</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>Phạm vi bày lá</x:v>
+        <x:v>Container có các lá con; không đồng nhất với Field</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>Ghi Area khi nhìn thấy</x:v>
+        <x:v>Ghi khi lá Home lần đầu hiện</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>Owner chốt loại; tên fixture</x:v>
+        <x:v>Owner chốt hierarchy · CG-35/36</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>Tên và ranh giới Home/Farm chưa khóa thành
-identity sản phẩm</x:v>
+        <x:v>Các lá Home khác trong V0 và quan hệ nhãn Region/Area còn mở</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-27, UI-30, UI-37</x:v>
+        <x:v>Decision 09 · CG-35–37; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
@@ -510,7 +529,7 @@
         <x:v>Area</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>Thuộc World; rộng hơn Rìa Rừng</x:v>
+        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>Khi người chơi nhìn thấy Area rừng</x:v>
@@ -532,7 +551,7 @@
         <x:v>Owner chốt loại; tên còn mở</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>Chưa có tên identity hiển thị cuối</x:v>
+        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
       </x:c>
       <x:c r="K9" s="9" t="str">
         <x:v>Decision 09 §10 · CG-01, UI-28–30</x:v>
@@ -546,16 +565,16 @@
         <x:v>Area</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Thuộc World</x:v>
+        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>Khi Area River được nhìn thấy</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Chứa exact Catch opportunity</x:v>
+        <x:v>Chứa 3 Fishing Spot giống nhau; Cast mỗi spot 1 AP</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Scroll/focus không là travel action</x:v>
+        <x:v>Scroll/focus không là travel action; Sleep làm mới ba spot</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
         <x:v>Phạm vi bày lá</x:v>
@@ -567,11 +586,10 @@
         <x:v>Owner chốt loại; tên làm việc</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>Tên hiển thị cuối chưa khóa</x:v>
+        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-27, UI-30; Mine/Fishing
-01</x:v>
+        <x:v>Decision 09 · CG-18/22–24; Fishing contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -582,7 +600,7 @@
         <x:v>Area</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>Thuộc World</x:v>
+        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
         <x:v>Khi Area Mine được nhìn thấy</x:v>
@@ -603,7 +621,7 @@
         <x:v>Owner chốt Mine · CG-17/20</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>Save qua reload và cấp Tool sau chưa triển khai/chốt</x:v>
+        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
       </x:c>
       <x:c r="K11" s="9" t="str">
         <x:v>Decision 09 · CG-17/19/20; Mine contract 01</x:v>
@@ -617,7 +635,7 @@
         <x:v>Area</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>Thuộc World</x:v>
+        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>Khi Area Commerce được nhìn thấy</x:v>
@@ -638,7 +656,7 @@
         <x:v>Owner chốt loại; tên làm việc</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>Tên hiển thị cuối chưa khóa</x:v>
+        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
       </x:c>
       <x:c r="K12" s="9" t="str">
         <x:v>Decision 09 §10 · UI-19, UI-27, UI-30</x:v>
@@ -696,7 +714,7 @@
         <x:v>Có trong khu nguồn khi lá được trình bày</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Ghép Pickaxe/Copper Pickaxe để Break; Rod để Cast; Herb để Gift</x:v>
+        <x:v>Ghép Pickaxe/Copper Pickaxe để Break; Rod để Cast lên Fishing Spot; Herb để Gift</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
         <x:v>Không bị tiêu khi dùng; đích thay đổi theo action</x:v>
@@ -714,43 +732,42 @@
         <x:v>Visual lá và vị trí chính xác trong hand chưa khóa</x:v>
       </x:c>
       <x:c r="K14" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-05–06, CG-17–20</x:v>
+        <x:v>Decision 09 · CG-05–06, CG-17–24</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="10" t="str">
-        <x:v>Tilled Soil</x:v>
+        <x:v>Tilled Soil (state)</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>Plot card</x:v>
+        <x:v>State of Soil; không là card identity</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>Plot trong Farm</x:v>
+        <x:v>Cùng lá Soil ở một vị trí Field</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>Hai plot mở đầu trong fixture giấy</x:v>
+        <x:v>Sau khi Hoe Till Soil trống, hoặc sau khi Harvest crop trên vị trí đó</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>Đích nhận một Seed hợp lệ</x:v>
+        <x:v>State Soil hợp lệ để nhận một Seed</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>Chính lá tại plot đổi identity thành crop theo
-giống</x:v>
+        <x:v>Hoe Till 1 AP đổi ảnh/state trong cùng Soil; Plant mới đổi identity sang Crop</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
-        <x:v>Đất đã cày</x:v>
+        <x:v>Đất đã cày; vẫn là Soil identity</x:v>
       </x:c>
       <x:c r="H15" s="9" t="str">
-        <x:v>Ghi khi lần đầu thấy plot</x:v>
+        <x:v>Không có entry riêng; Bách Khoa ghi identity Soil khi lá Soil hiện</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
-        <x:v>Owner chốt grammar</x:v>
+        <x:v>Owner sửa rõ chuyển trạng thái · CG-40</x:v>
       </x:c>
       <x:c r="J15" s="9" t="str">
-        <x:v>Số plot mở đầu là fixture giấy</x:v>
+        <x:v>Tên state giữ cho bộ lọc/tóm tắt; không là lá riêng</x:v>
       </x:c>
       <x:c r="K15" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-02, UI-02</x:v>
+        <x:v>Decision 09 · CG-02/34/40; Farm land contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" customHeight="1">
@@ -767,7 +784,7 @@
         <x:v>Có từ đầu; có thể Buy ở Supermarket</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Nguồn Plant lên Tilled Soil</x:v>
+        <x:v>Nguồn Plant lên Soil đã cày</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str">
         <x:v>Tiêu một Seed khi Plant; tạo Turnip Crop ở
@@ -797,18 +814,17 @@
         <x:v>Item · Crop</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>Cùng plot Farm sau Plant</x:v>
+        <x:v>Cùng ô đất trong Field sau Plant</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>Turnip Seed được Plant vào Tilled Soil</x:v>
+        <x:v>Turnip Seed được Plant vào Soil đã cày</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
         <x:v>Nhận Watering Can/Rain; Hand Harvest khi
 Mature</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
-        <x:v>Watered/Mature chỉ đổi state; Harvest trả plot
-về Soil và tạo Turnip item</x:v>
+        <x:v>Watered/Mature đổi state; Harvest trả vị trí về Soil đã cày và tạo Turnip item</x:v>
       </x:c>
       <x:c r="G17" s="9" t="str">
         <x:v>Growth, Watered, Mature qua visual</x:v>
@@ -923,15 +939,13 @@
         <x:v>Ghi khi Tool lần đầu hiện</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>Luật giấy V0</x:v>
+        <x:v>Owner chốt Watering Can thường V0 · CG-26</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
-        <x:v>CG-13: theo phạm vi/sức chứa bản gốc.
-Cần vị trí plot, vùng tưới và refill; art/sở hữu mở.</x:v>
+        <x:v>Một crop/1 AP; không nâng Can hoặc thêm refill trong V0. Art/sở hữu còn mở.</x:v>
       </x:c>
       <x:c r="K20" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-03–05, CG-13;
-Ore use reference 01 · §4.2, §7</x:v>
+        <x:v>Decision 09 · UI-03–05, CG-26; Farm land contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="62" customHeight="1">
@@ -948,11 +962,10 @@
         <x:v>Có khi Tool được sở hữu trong fixture V0</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Ghép Character, rồi lên exact Catch</x:v>
+        <x:v>Ghép Character rồi chạm Fishing Spot chưa spent để Cast</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
-        <x:v>Không tiêu Tool; nhận Fish khi Catch thành
-công</x:v>
+        <x:v>Không tiêu Tool; Cast 1 AP cho Fish hoặc No Bite; spot thành spent</x:v>
       </x:c>
       <x:c r="G21" s="9" t="str">
         <x:v>Được chọn / ghép nguồn</x:v>
@@ -961,15 +974,13 @@
         <x:v>Ghi khi Tool lần đầu hiện</x:v>
       </x:c>
       <x:c r="I21" s="9" t="str">
-        <x:v>Luật giấy V0</x:v>
+        <x:v>Owner chốt Fishing V0 · CG-24</x:v>
       </x:c>
       <x:c r="J21" s="9" t="str">
-        <x:v>Art/sở hữu chưa khóa; hoãn sửa fishing.
-Không mặc định Rod nâng bằng Ore.</x:v>
+        <x:v>Art/sở hữu và cấp nâng Rod còn mở</x:v>
       </x:c>
       <x:c r="K21" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-10, CG-10–11;
-Ore use reference 01 · §4–6</x:v>
+        <x:v>Decision 09 · CG-18/22–24; Fishing contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
@@ -1018,71 +1029,63 @@
         <x:v>River → Item</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Exact Catch phổ biến trong fixture giấy</x:v>
+        <x:v>Cast thành công trên một Fishing Spot chưa spent</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>Character + Rod lên Catch; Fish trong Item
-là nguồn gửi Shipping Bin</x:v>
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
-        <x:v>Catch nhận đúng Fish; xác nhận gửi Bin tiêu
-số lượng đã chọn, Gold trả cuối ngày</x:v>
+        <x:v>Nhận 1 Silver Minnow; gửi Bin tiêu số lượng đã chọn, Gold đến cuối ngày</x:v>
       </x:c>
       <x:c r="G23" s="9" t="str">
-        <x:v>Fresh khi nhận item</x:v>
+        <x:v>Fresh; số lượng trong Item</x:v>
       </x:c>
       <x:c r="H23" s="9" t="str">
-        <x:v>Ghi khi Fish lần đầu hiện; Catch đưa vào Item
-không thêm mục</x:v>
+        <x:v>Ghi khi Silver Minnow item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
       </x:c>
       <x:c r="I23" s="9" t="str">
-        <x:v>Owner chốt loại và bán · CG-10</x:v>
+        <x:v>Owner chốt Fish V0 · CG-24</x:v>
       </x:c>
       <x:c r="J23" s="9" t="str">
-        <x:v>Giá bán chưa chốt; cải thiện fishing để sau.
-Fixture chưa triển khai bán Fish.</x:v>
+        <x:v>Giá bán thuộc Commerce; art và runtime chưa triển khai</x:v>
       </x:c>
       <x:c r="K23" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-06, CG-10, UI-10, UI-21–22</x:v>
+        <x:v>Decision 09 · CG-10/18/22–24; Fishing contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>Blue Eel</x:v>
+        <x:v>Fishing Spot</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>Item · Fish</x:v>
+        <x:v>Source card</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>River → Item</x:v>
+        <x:v>River tableau</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>Exact Catch khi Rain trong fixture giấy</x:v>
+        <x:v>3 instance mở sẵn/ngày; odds ẩn 25/50/75 xáo ở Sleep</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>Character + Rod lên Catch khi Rain; Fish
-trong Item là nguồn gửi Shipping Bin</x:v>
+        <x:v>Character + Fishing Rod → Cast 1 AP; mỗi spot một lần/ngày</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
-        <x:v>Catch nhận đúng Fish; xác nhận gửi Bin tiêu
-số lượng đã chọn, Gold trả cuối ngày</x:v>
+        <x:v>Thành công: 1 Silver Minnow; No Bite: không Fish; cả hai làm spot spent</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>Fresh khi nhận item</x:v>
+        <x:v>Ready/spent; odds ẩn giữ suốt ngày</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
-        <x:v>Ghi khi Fish lần đầu hiện; Catch đưa vào Item
-không thêm mục</x:v>
+        <x:v>Ghi Fishing Spot khi identity lần đầu hiện</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>Owner chốt loại và bán · CG-10</x:v>
+        <x:v>Owner chốt Fishing V0 · CG-24</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
-        <x:v>Giá bán chưa chốt; cải thiện fishing để sau.
-Fixture chưa triển khai bán Fish.</x:v>
+        <x:v>Art cuối và save qua reload chưa triển khai</x:v>
       </x:c>
       <x:c r="K24" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-06, CG-10, UI-10, UI-21–22</x:v>
+        <x:v>Decision 09 · CG-18/22–24; Fishing contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
@@ -1307,7 +1310,7 @@
         <x:v>Equipment card · Thiết bị</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>Home/Farm tableau</x:v>
+        <x:v>Lá ở tableau Home; ngoài sức chứa đất Field</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
         <x:v>Có trong fixture vòng đầu</x:v>
@@ -1331,7 +1334,7 @@
         <x:v>Art/hiển thị hàng chờ cuối chưa khóa</x:v>
       </x:c>
       <x:c r="K31" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-09, UI-21–22</x:v>
+        <x:v>Decision 09 · CG-09/35/36, UI-21–22</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -1342,22 +1345,22 @@
         <x:v>Building card</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>Farm Area</x:v>
+        <x:v>Building card ở Home; chứa TV và Bed</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>Hiện ở Farm khi người chơi thấy Building</x:v>
+        <x:v>Khi chơi Home và lá Farmhouse hiện</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>Chạm Farmhouse mở TV bên trong; mở 0 AP navigation</x:v>
+        <x:v>Chạm Farmhouse mở tableau bên trong có TV và Bed</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
         <x:v>Chỉ mở nội dung; TV mới commit xem dự báo</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>Building có sub-card TV</x:v>
+        <x:v>Container Building; TV/Bed là lá con</x:v>
       </x:c>
       <x:c r="H32" s="9" t="str">
-        <x:v>Ghi Farmhouse khi thấy lá; ghi TV khi TV hiện</x:v>
+        <x:v>Ghi Farmhouse khi thấy lá; ghi TV/Bed khi từng lá hiện</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
         <x:v>Owner chốt grammar</x:v>
@@ -1366,7 +1369,7 @@
         <x:v>Art và bố cục bên trong Building chưa chốt</x:v>
       </x:c>
       <x:c r="K32" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-07/FH-01, UI-33</x:v>
+        <x:v>Decision 09 · CG-07/35/36, UI-33</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
@@ -1377,7 +1380,7 @@
         <x:v>Equipment card · Thiết bị</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>Bên trong Farmhouse</x:v>
+        <x:v>Lá con bên trong Farmhouse; ngoài sức chứa Field</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
         <x:v>Khi nội dung Farmhouse được mở</x:v>
@@ -1401,7 +1404,7 @@
         <x:v>Chức năng TV về sau không thuộc V0</x:v>
       </x:c>
       <x:c r="K33" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-09, UI-33</x:v>
+        <x:v>Decision 09 · CG-09/27, UI-33</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -1440,10 +1443,255 @@
         <x:v>Decision 09 §10 · UI-23–24, UI-31–32, UI-37</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="15" t="str">
+        <x:v>Soil</x:v>
+      </x:c>
+      <x:c r="B35" s="16" t="str">
+        <x:v>Plot card</x:v>
+      </x:c>
+      <x:c r="C35" s="16" t="str">
+        <x:v>Một vị trí đất trong Field</x:v>
+      </x:c>
+      <x:c r="D35" s="16" t="str">
+        <x:v>2 Soil trống + 3 Soil có bụi lúc đầu; xuất hiện thêm khi lá đá được Clear</x:v>
+      </x:c>
+      <x:c r="E35" s="16" t="str">
+        <x:v>Sickle Clear bụi 1 AP; Hoe Till Soil trống 1 AP</x:v>
+      </x:c>
+      <x:c r="F35" s="16" t="str">
+        <x:v>Dọn bụi và Till chỉ đổi ảnh/state cùng Soil; Plant mới đổi identity thành Crop</x:v>
+      </x:c>
+      <x:c r="G35" s="16" t="str">
+        <x:v>State: có bụi, đất trống hoặc đã cày; một vị trí đất</x:v>
+      </x:c>
+      <x:c r="H35" s="16" t="str">
+        <x:v>Một entry Soil khi identity lần đầu hiện; đổi state không mở mục mới</x:v>
+      </x:c>
+      <x:c r="I35" s="16" t="str">
+        <x:v>Owner chốt Clear/Till · CG-39/40</x:v>
+      </x:c>
+      <x:c r="J35" s="16" t="str">
+        <x:v>Hoe Till chỉ hợp lệ trên Soil trống; 1 AP, không item</x:v>
+      </x:c>
+      <x:c r="K35" s="16" t="str">
+        <x:v>Decision 09 · CG-25/27/35–40; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="62" customHeight="1">
+      <x:c r="A36" s="15" t="str">
+        <x:v>Field Rock</x:v>
+      </x:c>
+      <x:c r="B36" s="16" t="str">
+        <x:v>Obstacle card · tên làm việc</x:v>
+      </x:c>
+      <x:c r="C36" s="16" t="str">
+        <x:v>Ba vị trí đất trong Field</x:v>
+      </x:c>
+      <x:c r="D36" s="16" t="str">
+        <x:v>Đúng 3 lá đá lúc bắt đầu</x:v>
+      </x:c>
+      <x:c r="E36" s="16" t="str">
+        <x:v>Hoe lên lá đá để Clear 1 AP</x:v>
+      </x:c>
+      <x:c r="F36" s="16" t="str">
+        <x:v>Lá đá rời vị trí; Soil đất trống thay vào đúng vị trí cũ; nhận 1 Stone Item</x:v>
+      </x:c>
+      <x:c r="G36" s="16" t="str">
+        <x:v>Lá vật cản riêng; không là ảnh/state của Soil</x:v>
+      </x:c>
+      <x:c r="H36" s="16" t="str">
+        <x:v>Ghi Field Rock khi lá lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I36" s="16" t="str">
+        <x:v>Owner sửa rõ lá đá bị thay thế · CG-39</x:v>
+      </x:c>
+      <x:c r="J36" s="16" t="str">
+        <x:v>Tên Field Rock là nhãn làm việc; phân biệt với Rock source trong Mine</x:v>
+      </x:c>
+      <x:c r="K36" s="16" t="str">
+        <x:v>Decision 09 · CG-38/39; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="62" customHeight="1">
+      <x:c r="A37" s="15" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B37" s="16" t="str">
+        <x:v>Container card; nhãn loại còn mở</x:v>
+      </x:c>
+      <x:c r="C37" s="16" t="str">
+        <x:v>Lá con của Home</x:v>
+      </x:c>
+      <x:c r="D37" s="16" t="str">
+        <x:v>Khi chơi Home và lá Field hiện</x:v>
+      </x:c>
+      <x:c r="E37" s="16" t="str">
+        <x:v>Chạm Field mở tableau đất/luống/crop và vật cản</x:v>
+      </x:c>
+      <x:c r="F37" s="16" t="str">
+        <x:v>Mở Field 0 AP navigation; mỗi lá đất có action/state riêng</x:v>
+      </x:c>
+      <x:c r="G37" s="16" t="str">
+        <x:v>Container: tối đa 8 vị trí đất, riêng với Home</x:v>
+      </x:c>
+      <x:c r="H37" s="16" t="str">
+        <x:v>Ghi Field khi lá hiện; lá đất ghi khi từng identity hiện</x:v>
+      </x:c>
+      <x:c r="I37" s="16" t="str">
+        <x:v>Owner ủy quyền chốt Field V0 · CG-35–39</x:v>
+      </x:c>
+      <x:c r="J37" s="16" t="str">
+        <x:v>V0: 2 Soil trống + 3 Soil có bụi + 3 Field Rock; Clear đá thay lá tại cùng vị trí</x:v>
+      </x:c>
+      <x:c r="K37" s="16" t="str">
+        <x:v>Decision 09 · CG-25/27/35–39; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="62" customHeight="1">
+      <x:c r="A38" s="15" t="str">
+        <x:v>Bed</x:v>
+      </x:c>
+      <x:c r="B38" s="16" t="str">
+        <x:v>Loại lá chưa chốt</x:v>
+      </x:c>
+      <x:c r="C38" s="16" t="str">
+        <x:v>Lá con bên trong Farmhouse</x:v>
+      </x:c>
+      <x:c r="D38" s="16" t="str">
+        <x:v>Khi người chơi mở Farmhouse và Bed hiện</x:v>
+      </x:c>
+      <x:c r="E38" s="16" t="str">
+        <x:v>Lá giường là đích tương tác trong nhà; action Sleep cần contract riêng</x:v>
+      </x:c>
+      <x:c r="F38" s="16" t="str">
+        <x:v>Chưa chốt thao tác/chi phí Sleep trên Bed; không tự sinh commit mới</x:v>
+      </x:c>
+      <x:c r="G38" s="16" t="str">
+        <x:v>State cụ thể chưa chốt</x:v>
+      </x:c>
+      <x:c r="H38" s="16" t="str">
+        <x:v>Ghi Bed khi lá lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I38" s="16" t="str">
+        <x:v>Owner nêu lá Bed trong hierarchy · CG-35</x:v>
+      </x:c>
+      <x:c r="J38" s="16" t="str">
+        <x:v>Loại lá, thao tác Sleep và thông số còn mở</x:v>
+      </x:c>
+      <x:c r="K38" s="16" t="str">
+        <x:v>Decision 09 · CG-35/37; World nested-card architecture 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="62" customHeight="1">
+      <x:c r="A39" s="15" t="str">
+        <x:v>Sickle</x:v>
+      </x:c>
+      <x:c r="B39" s="16" t="str">
+        <x:v>Tool card</x:v>
+      </x:c>
+      <x:c r="C39" s="16" t="str">
+        <x:v>Item / khu nguồn từ đầu V0</x:v>
+      </x:c>
+      <x:c r="D39" s="16" t="str">
+        <x:v>Có từ đầu để Clear bụi</x:v>
+      </x:c>
+      <x:c r="E39" s="16" t="str">
+        <x:v>Chọn Sickle rồi chạm Soil có bụi trong Field</x:v>
+      </x:c>
+      <x:c r="F39" s="16" t="str">
+        <x:v>Clear 1 AP; Soil đổi ảnh sang đất trống; không item; Tool không tiêu</x:v>
+      </x:c>
+      <x:c r="G39" s="16" t="str">
+        <x:v>Tool dùng lại; không nâng cấp trong luật Clear V0</x:v>
+      </x:c>
+      <x:c r="H39" s="16" t="str">
+        <x:v>Ghi khi Sickle lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I39" s="16" t="str">
+        <x:v>Owner chốt Tool/phí · CG-39</x:v>
+      </x:c>
+      <x:c r="J39" s="16" t="str">
+        <x:v>Nguồn Tool từ đầu là lựa chọn triển khai để có đích dùng ngay</x:v>
+      </x:c>
+      <x:c r="K39" s="16" t="str">
+        <x:v>Decision 09 · CG-39; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="62" customHeight="1">
+      <x:c r="A40" s="15" t="str">
+        <x:v>Hoe</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="str">
+        <x:v>Tool card</x:v>
+      </x:c>
+      <x:c r="C40" s="16" t="str">
+        <x:v>Item / khu nguồn từ đầu V0</x:v>
+      </x:c>
+      <x:c r="D40" s="16" t="str">
+        <x:v>Có từ đầu để Clear đá Field</x:v>
+      </x:c>
+      <x:c r="E40" s="16" t="str">
+        <x:v>Chọn Hoe rồi chạm Field Rock để Clear, hoặc Soil trống để Till</x:v>
+      </x:c>
+      <x:c r="F40" s="16" t="str">
+        <x:v>Clear đá 1 AP: thay bằng Soil trống, nhận 1 Stone; Till 1 AP: cùng Soil đổi state đã cày; Tool không tiêu</x:v>
+      </x:c>
+      <x:c r="G40" s="16" t="str">
+        <x:v>Tool dùng lại cho Clear đá và Till đất trống</x:v>
+      </x:c>
+      <x:c r="H40" s="16" t="str">
+        <x:v>Ghi khi Hoe lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I40" s="16" t="str">
+        <x:v>Owner chốt Tool Clear/Till · CG-39/40</x:v>
+      </x:c>
+      <x:c r="J40" s="16" t="str">
+        <x:v>Không Till Soil có bụi, đá, Soil đã cày hoặc Crop</x:v>
+      </x:c>
+      <x:c r="K40" s="16" t="str">
+        <x:v>Decision 09 · CG-39/40; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="62" customHeight="1">
+      <x:c r="A41" s="15" t="str">
+        <x:v>Stone</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="str">
+        <x:v>Item / material</x:v>
+      </x:c>
+      <x:c r="C41" s="16" t="str">
+        <x:v>Item sau khi Clear đá Field</x:v>
+      </x:c>
+      <x:c r="D41" s="16" t="str">
+        <x:v>Nhận 1 Stone khi Hoe Clear một Field Rock</x:v>
+      </x:c>
+      <x:c r="E41" s="16" t="str">
+        <x:v>Output vào Item/inventory sau Clear đá; công dụng hoãn đến giai đoạn đổ nội dung</x:v>
+      </x:c>
+      <x:c r="F41" s="16" t="str">
+        <x:v>Giữ Item Stone sau Clear; không tự sinh recipe, giá bán hoặc mục tiêu V0</x:v>
+      </x:c>
+      <x:c r="G41" s="16" t="str">
+        <x:v>Một Item identity riêng với Field Rock</x:v>
+      </x:c>
+      <x:c r="H41" s="16" t="str">
+        <x:v>Ghi khi Stone item lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I41" s="16" t="str">
+        <x:v>Owner chốt output · CG-39; hoãn công dụng · CG-41</x:v>
+      </x:c>
+      <x:c r="J41" s="16" t="str">
+        <x:v>Công dụng, giá bán và nguồn Stone khác xử lý khi đổ nội dung vào game</x:v>
+      </x:c>
+      <x:c r="K41" s="16" t="str">
+        <x:v>Decision 09 · CG-39/41; Farm land contract 01</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2b78a8691654cac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf8386cff3f4757"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add first playable prototype and settle Ink card UI
</commit_message>
<xml_diff>
--- a/docs/current/LITTLE-VALLEY-CARD-REGISTER-V0.xlsx
+++ b/docs/current/LITTLE-VALLEY-CARD-REGISTER-V0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lá bài V0" sheetId="1" r:id="R32ef8b336b3949e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lá bài V0" sheetId="1" r:id="Re408d558e86249c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -56,6 +56,22 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243247"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF243247"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -76,7 +92,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -120,6 +136,29 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -128,8 +167,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CardsV0" displayName="CardsV0" ref="A6:K41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:K41"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CardsV0" displayName="CardsV0" ref="A6:K84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:K84"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Identity / tên làm việc"/>
     <x:tableColumn id="2" name="Loại lá"/>
@@ -390,7 +429,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="4" t="str">
-        <x:v>Phạm vi: lá đang dùng trong vòng đầu. Không đưa tên đã bác bỏ hoặc Seed/crop chưa có nguồn vào danh sách lá hiện thời.</x:v>
+        <x:v>Phạm vi: lá giấy V0 đang có nguồn. CG-53 Bean/Balm; CG-55–57 Hedgerow/Berry; CG-58/63 cây thường, Wood/Sap/Hardwood; CG-59–61 sáu Fruit Tree, Sapling/quả; CG-64–67 River Fish mười loài. Giá cuối còn mở.</x:v>
       </x:c>
       <x:c r="B4" s="4"/>
       <x:c r="C4" s="4"/>
@@ -480,10 +519,10 @@
         <x:v>Owner chốt grammar</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>Danh sách Region V0 và nhãn loại Region/Area còn cần đồng bộ</x:v>
+        <x:v>World chứa đúng 5 Region V0; Nell chưa có Region xuất hiện cụ thể</x:v>
       </x:c>
       <x:c r="K7" s="9" t="str">
-        <x:v>Decision 09 · CG-35/37, UI-37; World nested-card architecture 01</x:v>
+        <x:v>Decision 09 · CG-35/37/43, UI-37; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
@@ -500,7 +539,7 @@
         <x:v>Khi chơi World và lá Home hiện trên tableau Region</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Chạm Home mở tableau chứa Field, Farmhouse, Shipping Bin</x:v>
+        <x:v>Chạm Home mở tableau chứa Field, Farm Pond, Farmhouse, Shipping Bin</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
         <x:v>Mở Home 0 AP navigation; lá con giữ state riêng</x:v>
@@ -515,46 +554,45 @@
         <x:v>Owner chốt hierarchy · CG-35/36</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>Các lá Home khác trong V0 và quan hệ nhãn Region/Area còn mở</x:v>
+        <x:v>Bố cục tableau Home và các lá thêm về sau còn mở</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:v>Decision 09 · CG-35–37; World nested-card architecture 01</x:v>
+        <x:v>Decision 09 · CG-35–37/43; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>Area rừng (chưa đặt tên)</x:v>
+        <x:v>Forest</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>Area</x:v>
+        <x:v>Region card</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
+        <x:v>Lá con trực tiếp của World</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Khi người chơi nhìn thấy Area rừng</x:v>
+        <x:v>Khi lá Forest hiện trên tableau Region của World</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>Chứa Wild Herb hiện trực tiếp</x:v>
+        <x:v>Bày Hedgerow và bốn cây thường Oak/Maple/Pine/Mahogany; Wild Herb hiện trực tiếp theo nhịp riêng; không có lá Rìa Rừng</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Rìa Rừng chỉ là tên bối cảnh, không tạo lá
-riêng</x:v>
+        <x:v>Mở Forest 0 AP navigation; Rìa Rừng chỉ là bối cảnh</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>Phạm vi bày lá</x:v>
+        <x:v>Container; Wild Herb giữ cadence và state riêng</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>Ghi Area khi nhìn thấy</x:v>
+        <x:v>Ghi Forest khi chính lá Region lần đầu hiện; không tự ghi lá con</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>Owner chốt loại; tên còn mở</x:v>
+        <x:v>Owner chốt taxonomy · CG-43</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
+        <x:v>Bố cục/visual tableau Region còn mở; luật lá con theo contract riêng</x:v>
       </x:c>
       <x:c r="K9" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-01, UI-28–30</x:v>
+        <x:v>Decision 09 · CG-01/43, UI-28–30; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
@@ -562,34 +600,34 @@
         <x:v>River</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Area</x:v>
+        <x:v>Region card</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
+        <x:v>Lá con trực tiếp của World</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Khi Area River được nhìn thấy</x:v>
+        <x:v>Khi lá River hiện trên tableau Region của World</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Chứa 3 Fishing Spot giống nhau; Cast mỗi spot 1 AP</x:v>
+        <x:v>Chứa 3 Fishing Spot giống nhau; Nell hiện ngày 6/12/18 mỗi Season S18, ngoài ba spot</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
         <x:v>Scroll/focus không là travel action; Sleep làm mới ba spot</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>Phạm vi bày lá</x:v>
+        <x:v>Container; ba odds/spot độc lập với sự hiện diện của Nell</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>Ghi Area khi nhìn thấy</x:v>
+        <x:v>Ghi River khi chính lá Region lần đầu hiện; không tự ghi lá con</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>Owner chốt loại; tên làm việc</x:v>
+        <x:v>Owner chốt taxonomy · CG-43</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
+        <x:v>Bố cục/visual tableau Region còn mở; luật lá con theo contract riêng</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>Decision 09 · CG-18/22–24; Fishing contract 01</x:v>
+        <x:v>Decision 09 · CG-18/22–24/43/45–47; Fishing contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -597,34 +635,34 @@
         <x:v>Mine</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>Area</x:v>
+        <x:v>Region card</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
+        <x:v>Lá con trực tiếp của World</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Khi Area Mine được nhìn thấy</x:v>
+        <x:v>Khi lá Mine hiện trên tableau Region của World</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
         <x:v>Chứa 3 nguồn Rock/Ore Rock mở sẵn; Next từng ô; Descend khi lộ lối</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>Depth là status; Sleep/rời Area giữ tầng và vòng; Descend tạo tầng mới</x:v>
+        <x:v>Depth là status; Sleep/rời Mine giữ tầng và vòng; Descend tạo tầng mới</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
         <x:v>Tầng, 3 ô, vòng Next, route và nguồn spent</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>Ghi Area khi nhìn thấy</x:v>
+        <x:v>Ghi Mine khi chính lá Region lần đầu hiện; không tự ghi lá con</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>Owner chốt Mine · CG-17/20</x:v>
+        <x:v>Owner chốt taxonomy · CG-43</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
+        <x:v>Bố cục/visual tableau Region còn mở; luật lá con theo contract riêng</x:v>
       </x:c>
       <x:c r="K11" s="9" t="str">
-        <x:v>Decision 09 · CG-17/19/20; Mine contract 01</x:v>
+        <x:v>Decision 09 · CG-17/19/20/43; Mine contract 01</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -632,13 +670,13 @@
         <x:v>Commerce</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>Area</x:v>
+        <x:v>Region card</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>Lá con của World; vai trò Region/Area cần đồng bộ</x:v>
+        <x:v>Lá con trực tiếp của World</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Khi Area Commerce được nhìn thấy</x:v>
+        <x:v>Khi lá Commerce hiện trên tableau Region của World</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
         <x:v>Chứa Supermarket trong fixture V0</x:v>
@@ -650,16 +688,16 @@
         <x:v>Phạm vi bày lá</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>Ghi Area khi nhìn thấy</x:v>
+        <x:v>Ghi Commerce khi chính lá Region lần đầu hiện; không tự ghi lá con</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>Owner chốt loại; tên làm việc</x:v>
+        <x:v>Owner chốt taxonomy · CG-43</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>Vị trí trong tableau Region và nhãn loại Region/Area cần chốt</x:v>
+        <x:v>Bố cục/visual tableau Region còn mở; luật lá con theo contract riêng</x:v>
       </x:c>
       <x:c r="K12" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-19, UI-27, UI-30</x:v>
+        <x:v>Decision 09 · CG-09/43, UI-19/27/30; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
@@ -676,8 +714,7 @@
         <x:v>Có trong khu nguồn khi lá được trình bày</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Nguồn cho Harvest crop Mature và Collect Wild
-Herb</x:v>
+        <x:v>Nguồn cho Harvest crop Mature, Fruit Tree Có quả và Collect Wild Herb</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
         <x:v>Không bị tiêu khi dùng; đích thay đổi theo
@@ -701,39 +738,17 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
-      <x:c r="A14" s="10" t="str">
-        <x:v>Character</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="str">
-        <x:v>Person card</x:v>
-      </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>Khu nguồn / hand người chơi</x:v>
-      </x:c>
-      <x:c r="D14" s="9" t="str">
-        <x:v>Có trong khu nguồn khi lá được trình bày</x:v>
-      </x:c>
-      <x:c r="E14" s="9" t="str">
-        <x:v>Ghép Pickaxe/Copper Pickaxe để Break; Rod để Cast lên Fishing Spot; Herb để Gift</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="str">
-        <x:v>Không bị tiêu khi dùng; đích thay đổi theo action</x:v>
-      </x:c>
-      <x:c r="G14" s="9" t="str">
-        <x:v>Được chọn / ghép nguồn</x:v>
-      </x:c>
-      <x:c r="H14" s="9" t="str">
-        <x:v>Mục riêng khi lá lần đầu hiện</x:v>
-      </x:c>
-      <x:c r="I14" s="9" t="str">
-        <x:v>Owner chốt loại · Person</x:v>
-      </x:c>
-      <x:c r="J14" s="9" t="str">
-        <x:v>Visual lá và vị trí chính xác trong hand chưa khóa</x:v>
-      </x:c>
-      <x:c r="K14" s="9" t="str">
-        <x:v>Decision 09 · CG-05–06, CG-17–24</x:v>
-      </x:c>
+      <x:c r="A14" s="10"/>
+      <x:c r="B14" s="9"/>
+      <x:c r="C14" s="9"/>
+      <x:c r="D14" s="9"/>
+      <x:c r="E14" s="9"/>
+      <x:c r="F14" s="9"/>
+      <x:c r="G14" s="9"/>
+      <x:c r="H14" s="9"/>
+      <x:c r="I14" s="9"/>
+      <x:c r="J14" s="9"/>
+      <x:c r="K14" s="9"/>
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="10" t="str">
@@ -885,13 +900,13 @@
         <x:v>Item · Crop</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>Area rừng → Item</x:v>
+        <x:v>Forest → Item</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
         <x:v>Một Herb hiện trực tiếp theo cadence giấy</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Hand Collect; item dùng để Gift Nell</x:v>
+        <x:v>Hand Collect → Item; đúng Wild Herb item dùng Gift Nell V0</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
         <x:v>Giữ cùng identity khi đổi nơi; Gift tiêu item</x:v>
@@ -900,17 +915,16 @@
         <x:v>Hiện ở world hoặc số lượng Item</x:v>
       </x:c>
       <x:c r="H19" s="9" t="str">
-        <x:v>Ghi khi lá lần đầu hiện ở Area hoặc Item;
-Collect không thêm mục</x:v>
+        <x:v>Ghi khi lá lần đầu hiện ở Forest hoặc Item; Collect không thêm mục</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
         <x:v>Owner chốt loại · Crop</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
-        <x:v>Nhãn Forage cũ bị thay thế; cadence xuất hiện là fixture giấy</x:v>
+        <x:v>Forage là nhãn cũ; cadence nguồn còn là luật giấy, không đổi vì CG-49</x:v>
       </x:c>
       <x:c r="K19" s="9" t="str">
-        <x:v>Decision 09 §10 · CG-04, CG-06, UI-09</x:v>
+        <x:v>Decision 09 §10 · CG-04/06/43/49, UI-09; Nell Gift audit 04</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -927,22 +941,22 @@
         <x:v>Có khi Tool được sở hữu trong fixture V0</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Nguồn Water một Growing Crop hợp lệ</x:v>
+        <x:v>Nguồn Water một Growing Crop hợp lệ; chạm Farm Pond để múc nước</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>Không tiêu Tool; crop đổi visual Watered</x:v>
+        <x:v>Không tiêu Tool; Water dùng một lượng nước và crop đổi visual Watered; Pond nạp Can đầy 0 AP</x:v>
       </x:c>
       <x:c r="G20" s="9" t="str">
-        <x:v>Được chọn; không tạo identity Watered</x:v>
+        <x:v>Được chọn; lượng nước còn trong Can; không tạo identity Watered</x:v>
       </x:c>
       <x:c r="H20" s="9" t="str">
         <x:v>Ghi khi Tool lần đầu hiện</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>Owner chốt Watering Can thường V0 · CG-26</x:v>
+        <x:v>Owner chốt Can thường · CG-26; bổ sung nguồn nước · CG-69</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
-        <x:v>Một crop/1 AP; không nâng Can hoặc thêm refill trong V0. Art/sở hữu còn mở.</x:v>
+        <x:v>Một crop/1 AP; không nâng Can V0. Sức chứa 40 trong prototype là fixture; art/sở hữu còn mở.</x:v>
       </x:c>
       <x:c r="K20" s="9" t="str">
         <x:v>Decision 09 · UI-03–05, CG-26; Farm land contract 01</x:v>
@@ -1029,7 +1043,7 @@
         <x:v>River → Item</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Cast thành công trên một Fishing Spot chưa spent</x:v>
+        <x:v>Cast thành công và rút trúng Silver Minnow từ tập Fish đủ Season</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
@@ -1070,7 +1084,7 @@
         <x:v>Character + Fishing Rod → Cast 1 AP; mỗi spot một lần/ngày</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
-        <x:v>Thành công: 1 Silver Minnow; No Bite: không Fish; cả hai làm spot spent</x:v>
+        <x:v>Thành công: rút đều 1 Fish đủ Season/Today Weather/pha (CG-64–67); No Bite: không Fish; spot spent cả hai. Next Phase không hồi spot/đổi odds</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
         <x:v>Ready/spent; odds ẩn giữ suốt ngày</x:v>
@@ -1085,7 +1099,7 @@
         <x:v>Art cuối và save qua reload chưa triển khai</x:v>
       </x:c>
       <x:c r="K24" s="9" t="str">
-        <x:v>Decision 09 · CG-18/22–24; Fishing contract 01</x:v>
+        <x:v>Decision 09 · CG-18/22–24/64–67; Fishing contract 01; River Fish batch 04</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
@@ -1236,34 +1250,31 @@
         <x:v>Person card</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>World khi có lịch; khu Person sau sở hữu</x:v>
+        <x:v>River khi có lịch; khu Person sau sở hữu</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>Lá world hiện theo lịch; control ability khi
-đã sở hữu</x:v>
+        <x:v>World card hiện trọn ngày 6/12/18 mỗi Season S18 trong River; control ability sau sở hữu</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Nhận Character + Herb để Gift; control kích
-hoạt ability</x:v>
+        <x:v>Character + Wild Herb item → Gift 1 AP gốc nếu Heart dưới cap; control ability</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>Gift đầu sở hữu và nhận Heart; ability tiêu
-Heart tạo AP relief</x:v>
+        <x:v>Gift đầu sở hữu Nell; mỗi Gift hợp lệ +1 Nell Heart; ability tiêu 1 Heart → 2 AP relief</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>Owned, Heart, Gift/ability hôm nay</x:v>
+        <x:v>Owned, Nell Heart 0–2 (cap 2), Gift/ability hôm nay</x:v>
       </x:c>
       <x:c r="H29" s="9" t="str">
         <x:v>Một mục identity khi Nell lần đầu hiện</x:v>
       </x:c>
       <x:c r="I29" s="9" t="str">
-        <x:v>Owner chốt grammar</x:v>
+        <x:v>Owner chốt Season đầu · CG-46; Season sau/Gift item/Gift số/cap Nell là chuyển thể CG-47/49–51</x:v>
       </x:c>
       <x:c r="J29" s="9" t="str">
-        <x:v>Lịch, sở thích Gift và icon cuối là fixture</x:v>
+        <x:v>Art, cân bằng phát hành và lịch nếu Season khác S18 còn mở; cap Person khác chưa chọn</x:v>
       </x:c>
       <x:c r="K29" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-13–18</x:v>
+        <x:v>Decision 09 · UI-13–18, CG-45–51; Person/Heart decisions; Nell checks 01–06</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -1409,7 +1420,7 @@
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
       <x:c r="A34" s="10" t="str">
-        <x:v>Bách Khoa Thung Lũng</x:v>
+        <x:v>Valley Almanac</x:v>
       </x:c>
       <x:c r="B34" s="9" t="str">
         <x:v>Utility card</x:v>
@@ -1437,10 +1448,10 @@
         <x:v>Owner chốt grammar</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
-        <x:v>Nhóm/lọc và độ sâu entry còn mở</x:v>
+        <x:v>English display name per UI-47; grouping and entry depth remain open</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
-        <x:v>Decision 09 §10 · UI-23–24, UI-31–32, UI-37</x:v>
+        <x:v>Decision 09 §10 · UI-23–24, UI-31–32, UI-37, UI-47</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
@@ -1460,7 +1471,7 @@
         <x:v>Sickle Clear bụi 1 AP; Hoe Till Soil trống 1 AP</x:v>
       </x:c>
       <x:c r="F35" s="16" t="str">
-        <x:v>Dọn bụi và Till chỉ đổi ảnh/state cùng Soil; Plant mới đổi identity thành Crop</x:v>
+        <x:v>Dọn bụi và Till chỉ đổi ảnh/state cùng Soil; Plant crop hoặc Fruit Tree thay identity tại cùng vị trí</x:v>
       </x:c>
       <x:c r="G35" s="16" t="str">
         <x:v>State: có bụi, đất trống hoặc đã cày; một vị trí đất</x:v>
@@ -1527,7 +1538,7 @@
         <x:v>Khi chơi Home và lá Field hiện</x:v>
       </x:c>
       <x:c r="E37" s="16" t="str">
-        <x:v>Chạm Field mở tableau đất/luống/crop và vật cản</x:v>
+        <x:v>Chạm Field mở tableau tám vị trí Soil/crop/Fruit Tree/vật cản</x:v>
       </x:c>
       <x:c r="F37" s="16" t="str">
         <x:v>Mở Field 0 AP navigation; mỗi lá đất có action/state riêng</x:v>
@@ -1553,34 +1564,34 @@
         <x:v>Bed</x:v>
       </x:c>
       <x:c r="B38" s="16" t="str">
-        <x:v>Loại lá chưa chốt</x:v>
+        <x:v>Equipment card · Thiết bị</x:v>
       </x:c>
       <x:c r="C38" s="16" t="str">
         <x:v>Lá con bên trong Farmhouse</x:v>
       </x:c>
       <x:c r="D38" s="16" t="str">
-        <x:v>Khi người chơi mở Farmhouse và Bed hiện</x:v>
+        <x:v>Khi mở tableau Farmhouse và chính lá Bed hiện</x:v>
       </x:c>
       <x:c r="E38" s="16" t="str">
-        <x:v>Lá giường là đích tương tác trong nhà; action Sleep cần contract riêng</x:v>
+        <x:v>Chạm Bed trực tiếp để thực hiện Sleep; không cần nguồn hoặc lớp Bed riêng</x:v>
       </x:c>
       <x:c r="F38" s="16" t="str">
-        <x:v>Chưa chốt thao tác/chi phí Sleep trên Bed; không tự sinh commit mới</x:v>
+        <x:v>Sleep chuyển sang ngày mới theo luật ngày hiện hành; mở Farmhouse chỉ là navigation 0 AP</x:v>
       </x:c>
       <x:c r="G38" s="16" t="str">
-        <x:v>State cụ thể chưa chốt</x:v>
+        <x:v>Không chốt state riêng trên Bed; ngày mới xử lý theo các contract cơ chế</x:v>
       </x:c>
       <x:c r="H38" s="16" t="str">
         <x:v>Ghi Bed khi lá lần đầu hiện</x:v>
       </x:c>
       <x:c r="I38" s="16" t="str">
-        <x:v>Owner nêu lá Bed trong hierarchy · CG-35</x:v>
+        <x:v>Owner chốt loại và đường Sleep · CG-44</x:v>
       </x:c>
       <x:c r="J38" s="16" t="str">
-        <x:v>Loại lá, thao tác Sleep và thông số còn mở</x:v>
+        <x:v>Visual Bed và phản hồi chuyển ngày còn mở; không thêm thông số AP trong quyết định này</x:v>
       </x:c>
       <x:c r="K38" s="16" t="str">
-        <x:v>Decision 09 · CG-35/37; World nested-card architecture 01</x:v>
+        <x:v>Decision 09 · CG-35/37/44; World nested-card architecture 01</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1688,10 +1699,1550 @@
         <x:v>Decision 09 · CG-39/41; Farm land contract 01</x:v>
       </x:c>
     </x:row>
+    <x:row r="42" ht="62" customHeight="1">
+      <x:c r="A42" s="15" t="str">
+        <x:v>Runner Bean Seed</x:v>
+      </x:c>
+      <x:c r="B42" s="16" t="str">
+        <x:v>Item / Seed</x:v>
+      </x:c>
+      <x:c r="C42" s="16" t="str">
+        <x:v>Item; cùng identity trên thẻ hàng shop</x:v>
+      </x:c>
+      <x:c r="D42" s="16" t="str">
+        <x:v>Supermarket niêm yết trong Season giấy đầu; nhận vào Item khi Buy</x:v>
+      </x:c>
+      <x:c r="E42" s="16" t="str">
+        <x:v>Nguồn Plant lên một Soil đã cày trong Field</x:v>
+      </x:c>
+      <x:c r="F42" s="16" t="str">
+        <x:v>Buy 0 AP dùng Gold hiện có; Plant 1 AP tiêu Seed và tạo Runner Bean Crop</x:v>
+      </x:c>
+      <x:c r="G42" s="16" t="str">
+        <x:v>Số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H42" s="16" t="str">
+        <x:v>Ghi khi Seed hiện trong shop panel, dù chưa Buy</x:v>
+      </x:c>
+      <x:c r="I42" s="16" t="str">
+        <x:v>Tên Crop chủ dự án chọn; nguồn Seed là chuyển thể CG-53</x:v>
+      </x:c>
+      <x:c r="J42" s="16" t="str">
+        <x:v>Giá/Season sau còn mở; không có thưởng Seed từ Bách Khoa</x:v>
+      </x:c>
+      <x:c r="K42" s="16" t="str">
+        <x:v>Crop identity audit 20; Decision 09 · CG-53/UI-23/37; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="62" customHeight="1">
+      <x:c r="A43" s="15" t="str">
+        <x:v>Runner Bean Crop</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="str">
+        <x:v>Item · Crop</x:v>
+      </x:c>
+      <x:c r="C43" s="16" t="str">
+        <x:v>Cùng một vị trí Soil trong Field sau Plant</x:v>
+      </x:c>
+      <x:c r="D43" s="16" t="str">
+        <x:v>Runner Bean Seed được Plant vào Soil đã cày</x:v>
+      </x:c>
+      <x:c r="E43" s="16" t="str">
+        <x:v>Watering Can/Rain khi Growing; Hand khi Mature</x:v>
+      </x:c>
+      <x:c r="F43" s="16" t="str">
+        <x:v>Watered tăng growth tại Sleep; Harvest trả plot về Soil đã cày và tạo Runner Bean item</x:v>
+      </x:c>
+      <x:c r="G43" s="16" t="str">
+        <x:v>Growth, Watered, Mature trên chính lá Crop</x:v>
+      </x:c>
+      <x:c r="H43" s="16" t="str">
+        <x:v>Mục riêng khi Crop lần đầu hiện ở Field</x:v>
+      </x:c>
+      <x:c r="I43" s="16" t="str">
+        <x:v>Identity theo grammar CG-02/40; profile giấy CG-53</x:v>
+      </x:c>
+      <x:c r="J43" s="16" t="str">
+        <x:v>Nhịp growth/yield là fixture; không tự thêm regrow hoặc trellis</x:v>
+      </x:c>
+      <x:c r="K43" s="16" t="str">
+        <x:v>Decision 09 · CG-02/40/53; Farm grammar 41; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="62" customHeight="1">
+      <x:c r="A44" s="15" t="str">
+        <x:v>Runner Bean</x:v>
+      </x:c>
+      <x:c r="B44" s="16" t="str">
+        <x:v>Item · Crop</x:v>
+      </x:c>
+      <x:c r="C44" s="16" t="str">
+        <x:v>Item sau Harvest</x:v>
+      </x:c>
+      <x:c r="D44" s="16" t="str">
+        <x:v>Hand Harvest Runner Bean Crop Mature</x:v>
+      </x:c>
+      <x:c r="E44" s="16" t="str">
+        <x:v>Giữ trong Item hoặc gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F44" s="16" t="str">
+        <x:v>Gửi Bin tiêu item; Gold chờ trả cuối ngày; không tự tạo Seed</x:v>
+      </x:c>
+      <x:c r="G44" s="16" t="str">
+        <x:v>Fresh và số lượng là thuộc tính</x:v>
+      </x:c>
+      <x:c r="H44" s="16" t="str">
+        <x:v>Mục riêng khi output lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I44" s="16" t="str">
+        <x:v>Tên Crop chủ dự án chọn; output giấy CG-53</x:v>
+      </x:c>
+      <x:c r="J44" s="16" t="str">
+        <x:v>Giá Sell và công dụng ngoài Keep/Sell còn mở; không là Gift Nell</x:v>
+      </x:c>
+      <x:c r="K44" s="16" t="str">
+        <x:v>Crop identity audit 20; Decision 09 · CG-49/53; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="62" customHeight="1">
+      <x:c r="A45" s="15" t="str">
+        <x:v>Lemon Balm Seed</x:v>
+      </x:c>
+      <x:c r="B45" s="16" t="str">
+        <x:v>Item / Seed</x:v>
+      </x:c>
+      <x:c r="C45" s="16" t="str">
+        <x:v>Item; cùng identity trên thẻ hàng shop</x:v>
+      </x:c>
+      <x:c r="D45" s="16" t="str">
+        <x:v>Supermarket niêm yết trong Season giấy đầu; nhận vào Item khi Buy</x:v>
+      </x:c>
+      <x:c r="E45" s="16" t="str">
+        <x:v>Nguồn Plant lên một Soil đã cày trong Field</x:v>
+      </x:c>
+      <x:c r="F45" s="16" t="str">
+        <x:v>Buy 0 AP dùng Gold hiện có; Plant 1 AP tiêu Seed và tạo Lemon Balm Crop</x:v>
+      </x:c>
+      <x:c r="G45" s="16" t="str">
+        <x:v>Số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H45" s="16" t="str">
+        <x:v>Ghi khi Seed hiện trong shop panel, dù chưa Buy</x:v>
+      </x:c>
+      <x:c r="I45" s="16" t="str">
+        <x:v>Tên Crop chủ dự án chọn; nguồn Seed là chuyển thể CG-53</x:v>
+      </x:c>
+      <x:c r="J45" s="16" t="str">
+        <x:v>Giá/Season sau còn mở; không có thưởng Seed từ Bách Khoa</x:v>
+      </x:c>
+      <x:c r="K45" s="16" t="str">
+        <x:v>Crop identity audit 20; Decision 09 · CG-53/UI-23/37; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="62" customHeight="1">
+      <x:c r="A46" s="15" t="str">
+        <x:v>Lemon Balm Crop</x:v>
+      </x:c>
+      <x:c r="B46" s="16" t="str">
+        <x:v>Item · Crop</x:v>
+      </x:c>
+      <x:c r="C46" s="16" t="str">
+        <x:v>Cùng một vị trí Soil trong Field sau Plant</x:v>
+      </x:c>
+      <x:c r="D46" s="16" t="str">
+        <x:v>Lemon Balm Seed được Plant vào Soil đã cày</x:v>
+      </x:c>
+      <x:c r="E46" s="16" t="str">
+        <x:v>Watering Can/Rain khi Growing; Hand khi Mature</x:v>
+      </x:c>
+      <x:c r="F46" s="16" t="str">
+        <x:v>Watered tăng growth tại Sleep; Harvest trả plot về Soil đã cày và tạo Lemon Balm item</x:v>
+      </x:c>
+      <x:c r="G46" s="16" t="str">
+        <x:v>Growth, Watered, Mature trên chính lá Crop</x:v>
+      </x:c>
+      <x:c r="H46" s="16" t="str">
+        <x:v>Mục riêng khi Crop lần đầu hiện ở Field</x:v>
+      </x:c>
+      <x:c r="I46" s="16" t="str">
+        <x:v>Identity theo grammar CG-02/40; profile giấy CG-53</x:v>
+      </x:c>
+      <x:c r="J46" s="16" t="str">
+        <x:v>Nhịp growth/yield là fixture; không tự thêm tác dụng Herb</x:v>
+      </x:c>
+      <x:c r="K46" s="16" t="str">
+        <x:v>Decision 09 · CG-02/40/53; Farm grammar 41; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="62" customHeight="1">
+      <x:c r="A47" s="15" t="str">
+        <x:v>Lemon Balm</x:v>
+      </x:c>
+      <x:c r="B47" s="16" t="str">
+        <x:v>Item · Crop · Herb subtype</x:v>
+      </x:c>
+      <x:c r="C47" s="16" t="str">
+        <x:v>Item sau Harvest</x:v>
+      </x:c>
+      <x:c r="D47" s="16" t="str">
+        <x:v>Hand Harvest Lemon Balm Crop Mature</x:v>
+      </x:c>
+      <x:c r="E47" s="16" t="str">
+        <x:v>Giữ trong Item hoặc gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F47" s="16" t="str">
+        <x:v>Gửi Bin tiêu item; Gold chờ trả cuối ngày; không tự tạo Seed</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="str">
+        <x:v>Fresh, Herb subtype và số lượng là thuộc tính</x:v>
+      </x:c>
+      <x:c r="H47" s="16" t="str">
+        <x:v>Mục riêng khi output lần đầu hiện</x:v>
+      </x:c>
+      <x:c r="I47" s="16" t="str">
+        <x:v>Tên Crop chủ dự án chọn; output giấy CG-53</x:v>
+      </x:c>
+      <x:c r="J47" s="16" t="str">
+        <x:v>Giá Sell/công dụng ngoài Keep/Sell còn mở; Nell chỉ nhận Wild Herb</x:v>
+      </x:c>
+      <x:c r="K47" s="16" t="str">
+        <x:v>Crop identity audit 20; Decision 09 · CG-49/53; Crop content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="62" customHeight="1">
+      <x:c r="A48" s="15" t="str">
+        <x:v>Hedgerow</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="str">
+        <x:v>Vegetation · bụi cây bám đất</x:v>
+      </x:c>
+      <x:c r="C48" s="16" t="str">
+        <x:v>Tableau Forest; bối cảnh Rìa Rừng</x:v>
+      </x:c>
+      <x:c r="D48" s="16" t="str">
+        <x:v>Bụi thường trực; Có quả từ đầu Season; giữ state qua Sleep/Back</x:v>
+      </x:c>
+      <x:c r="E48" s="16" t="str">
+        <x:v>Hand → chính lá bụi Có quả để hái Berry (Pick Berry)</x:v>
+      </x:c>
+      <x:c r="F48" s="16" t="str">
+        <x:v>Hái 1 AP gốc tạo 1 Hedgerow Berry trong Item; bụi ở lại và chuyển Đã hái</x:v>
+      </x:c>
+      <x:c r="G48" s="16" t="str">
+        <x:v>Có quả/Đã hái là state cùng identity; một Berry mỗi Season giấy</x:v>
+      </x:c>
+      <x:c r="H48" s="16" t="str">
+        <x:v>Ghi khi lá bụi lần đầu hiện trong Forest</x:v>
+      </x:c>
+      <x:c r="I48" s="16" t="str">
+        <x:v>CG-56: chủ dự án làm rõ bụi và hái; CG-57: bụi không là Item; nhịp là chuyển thể</x:v>
+      </x:c>
+      <x:c r="J48" s="16" t="str">
+        <x:v>Cùng nhóm Vegetation với cây lấy gỗ CG-58; bụi không vào Item; giá Berry chưa chốt</x:v>
+      </x:c>
+      <x:c r="K48" s="16" t="str">
+        <x:v>Decision 09 · CG-55–57; Forest content batch 01; Stardew Wiki Salmonberry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="62" customHeight="1">
+      <x:c r="A49" s="15" t="str">
+        <x:v>Hedgerow Berry</x:v>
+      </x:c>
+      <x:c r="B49" s="16" t="str">
+        <x:v>Item · Crop · Berry subtype</x:v>
+      </x:c>
+      <x:c r="C49" s="16" t="str">
+        <x:v>Item sau khi hái từ bụi Hedgerow</x:v>
+      </x:c>
+      <x:c r="D49" s="16" t="str">
+        <x:v>Nhận 1 Berry khi Hand hái bụi Hedgerow Có quả</x:v>
+      </x:c>
+      <x:c r="E49" s="16" t="str">
+        <x:v>Giữ trong Item hoặc gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F49" s="16" t="str">
+        <x:v>Bin tiêu item 0 AP; Gold chờ trả cuối ngày; không Plant/Gift Nell</x:v>
+      </x:c>
+      <x:c r="G49" s="16" t="str">
+        <x:v>Số lượng trong Item; item giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H49" s="16" t="str">
+        <x:v>Ghi khi lá Berry output lần đầu hiện trong Item</x:v>
+      </x:c>
+      <x:c r="I49" s="16" t="str">
+        <x:v>Tên giấy cũ; quan hệ bụi → quả làm rõ CG-56</x:v>
+      </x:c>
+      <x:c r="J49" s="16" t="str">
+        <x:v>2G chỉ là fixture kiểm đường Seed; giá/công dụng khác còn mở</x:v>
+      </x:c>
+      <x:c r="K49" s="16" t="str">
+        <x:v>Decision 09 · CG-06/49/55–57; Forest content batch 01</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="62" customHeight="1">
+      <x:c r="A50" s="19" t="str">
+        <x:v>Oak Tree</x:v>
+      </x:c>
+      <x:c r="B50" s="18" t="str">
+        <x:v>Vegetation · cây bám đất</x:v>
+      </x:c>
+      <x:c r="C50" s="18" t="str">
+        <x:v>Tableau Forest</x:v>
+      </x:c>
+      <x:c r="D50" s="18" t="str">
+        <x:v>Một lá Mature từ đầu; cây đã dọn trở lại Mature đầu Season kế</x:v>
+      </x:c>
+      <x:c r="E50" s="18" t="str">
+        <x:v>Axe → Oak Tree Mature hoặc Stump</x:v>
+      </x:c>
+      <x:c r="F50" s="18" t="str">
+        <x:v>Mature Chop 1 AP: 2 Wood + 1 Sap, thành Stump; Chop Stump 1 AP: +1 Wood, rời Forest</x:v>
+      </x:c>
+      <x:c r="G50" s="18" t="str">
+        <x:v>Mature / Stump / đã dọn; Sleep giữ state; Stump chưa dọn chặn hồi</x:v>
+      </x:c>
+      <x:c r="H50" s="18" t="str">
+        <x:v>Ghi khi lá cây lần đầu hiện ở Forest; Stump không có entry riêng</x:v>
+      </x:c>
+      <x:c r="I50" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-58</x:v>
+      </x:c>
+      <x:c r="J50" s="18" t="str">
+        <x:v>Một lá mỗi loài; seed, Moss, Tapper và sink Wood/Sap chưa chọn</x:v>
+      </x:c>
+      <x:c r="K50" s="18" t="str">
+        <x:v>Decision 09 · CG-58; Forest content batch 01; Stardew Wiki Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="62" customHeight="1">
+      <x:c r="A51" s="19" t="str">
+        <x:v>Maple Tree</x:v>
+      </x:c>
+      <x:c r="B51" s="18" t="str">
+        <x:v>Vegetation · cây bám đất</x:v>
+      </x:c>
+      <x:c r="C51" s="18" t="str">
+        <x:v>Tableau Forest</x:v>
+      </x:c>
+      <x:c r="D51" s="18" t="str">
+        <x:v>Một lá Mature từ đầu; cây đã dọn trở lại Mature đầu Season kế</x:v>
+      </x:c>
+      <x:c r="E51" s="18" t="str">
+        <x:v>Axe → Maple Tree Mature hoặc Stump</x:v>
+      </x:c>
+      <x:c r="F51" s="18" t="str">
+        <x:v>Mature Chop 1 AP: 2 Wood + 1 Sap, thành Stump; Chop Stump 1 AP: +1 Wood, rời Forest</x:v>
+      </x:c>
+      <x:c r="G51" s="18" t="str">
+        <x:v>Mature / Stump / đã dọn; Sleep giữ state; Stump chưa dọn chặn hồi</x:v>
+      </x:c>
+      <x:c r="H51" s="18" t="str">
+        <x:v>Ghi khi lá cây lần đầu hiện ở Forest; Stump không có entry riêng</x:v>
+      </x:c>
+      <x:c r="I51" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-58</x:v>
+      </x:c>
+      <x:c r="J51" s="18" t="str">
+        <x:v>Một lá mỗi loài; seed, Moss, Tapper và sink Wood/Sap chưa chọn</x:v>
+      </x:c>
+      <x:c r="K51" s="18" t="str">
+        <x:v>Decision 09 · CG-58; Forest content batch 01; Stardew Wiki Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="62" customHeight="1">
+      <x:c r="A52" s="19" t="str">
+        <x:v>Pine Tree</x:v>
+      </x:c>
+      <x:c r="B52" s="18" t="str">
+        <x:v>Vegetation · cây bám đất</x:v>
+      </x:c>
+      <x:c r="C52" s="18" t="str">
+        <x:v>Tableau Forest</x:v>
+      </x:c>
+      <x:c r="D52" s="18" t="str">
+        <x:v>Một lá Mature từ đầu; cây đã dọn trở lại Mature đầu Season kế</x:v>
+      </x:c>
+      <x:c r="E52" s="18" t="str">
+        <x:v>Axe → Pine Tree Mature hoặc Stump</x:v>
+      </x:c>
+      <x:c r="F52" s="18" t="str">
+        <x:v>Mature Chop 1 AP: 2 Wood + 1 Sap, thành Stump; Chop Stump 1 AP: +1 Wood, rời Forest</x:v>
+      </x:c>
+      <x:c r="G52" s="18" t="str">
+        <x:v>Mature / Stump / đã dọn; Sleep giữ state; Stump chưa dọn chặn hồi</x:v>
+      </x:c>
+      <x:c r="H52" s="18" t="str">
+        <x:v>Ghi khi lá cây lần đầu hiện ở Forest; Stump không có entry riêng</x:v>
+      </x:c>
+      <x:c r="I52" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-58</x:v>
+      </x:c>
+      <x:c r="J52" s="18" t="str">
+        <x:v>Một lá mỗi loài; seed, Moss, Tapper và sink Wood/Sap chưa chọn</x:v>
+      </x:c>
+      <x:c r="K52" s="18" t="str">
+        <x:v>Decision 09 · CG-58; Forest content batch 01; Stardew Wiki Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="62" customHeight="1">
+      <x:c r="A53" s="19" t="str">
+        <x:v>Axe</x:v>
+      </x:c>
+      <x:c r="B53" s="18" t="str">
+        <x:v>Tool card</x:v>
+      </x:c>
+      <x:c r="C53" s="18" t="str">
+        <x:v>Item / khu nguồn từ đầu V0</x:v>
+      </x:c>
+      <x:c r="D53" s="18" t="str">
+        <x:v>Có từ đầu V0 cùng các Tool khởi đầu</x:v>
+      </x:c>
+      <x:c r="E53" s="18" t="str">
+        <x:v>Chọn Axe rồi chạm Oak/Maple/Pine/Mahogany Mature hoặc Stump ở Forest; Fruit Tree Young hoặc Mature ở Field</x:v>
+      </x:c>
+      <x:c r="F53" s="18" t="str">
+        <x:v>Chop/Chop Stump Forest hoặc Chop Fruit Tree Field đều 1 AP gốc; Axe dùng lại, không tiêu</x:v>
+      </x:c>
+      <x:c r="G53" s="18" t="str">
+        <x:v>Nguồn Tool giữ qua các action</x:v>
+      </x:c>
+      <x:c r="H53" s="18" t="str">
+        <x:v>Ghi khi Axe lần đầu hiện trong Item</x:v>
+      </x:c>
+      <x:c r="I53" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-58/59–61/63</x:v>
+      </x:c>
+      <x:c r="J53" s="18" t="str">
+        <x:v>Cây ăn quả Field không để Stump; nâng cấp Tool để sau</x:v>
+      </x:c>
+      <x:c r="K53" s="18" t="str">
+        <x:v>Decision 09 · CG-58/59–61/63; Forest and Fruit Tree content batch 01; Stardew Wiki Axes/Trees/Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="62" customHeight="1">
+      <x:c r="A54" s="19" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="B54" s="18" t="str">
+        <x:v>Item / material</x:v>
+      </x:c>
+      <x:c r="C54" s="18" t="str">
+        <x:v>Item sau Chop/Chop Stump ở Forest hoặc Chop cây ăn quả Mature ở Field</x:v>
+      </x:c>
+      <x:c r="D54" s="18" t="str">
+        <x:v>Oak/Maple/Pine Mature Chop cho 2; Forest Stump Chop cho 1; Fruit Tree Mature Chop cho 2; Mahogany Mature cho Hardwood thay Wood</x:v>
+      </x:c>
+      <x:c r="E54" s="18" t="str">
+        <x:v>Output vào Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="F54" s="18" t="str">
+        <x:v>Chưa có recipe, giá bán, Bin hoặc Gift V0</x:v>
+      </x:c>
+      <x:c r="G54" s="18" t="str">
+        <x:v>Một identity Item; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H54" s="18" t="str">
+        <x:v>Ghi khi Wood item đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I54" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-58/59</x:v>
+      </x:c>
+      <x:c r="J54" s="18" t="str">
+        <x:v>Giá, công dụng và nguồn bổ sung của Wood để giai đoạn nội dung sau</x:v>
+      </x:c>
+      <x:c r="K54" s="18" t="str">
+        <x:v>Decision 09 · CG-58/59; Forest and Fruit Tree content batch 01; Stardew Wiki Trees/Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="62" customHeight="1">
+      <x:c r="A55" s="19" t="str">
+        <x:v>Sap</x:v>
+      </x:c>
+      <x:c r="B55" s="18" t="str">
+        <x:v>Item / material</x:v>
+      </x:c>
+      <x:c r="C55" s="18" t="str">
+        <x:v>Item sau Chop Oak/Maple/Pine/Mahogany Mature ở Forest</x:v>
+      </x:c>
+      <x:c r="D55" s="18" t="str">
+        <x:v>Chop Oak/Maple/Pine/Mahogany Mature cho 1 Sap; Stump không cho Sap trong V0</x:v>
+      </x:c>
+      <x:c r="E55" s="18" t="str">
+        <x:v>Output vào Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="F55" s="18" t="str">
+        <x:v>Chưa có recipe, giá bán, Bin hoặc Gift V0</x:v>
+      </x:c>
+      <x:c r="G55" s="18" t="str">
+        <x:v>Một identity Item; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H55" s="18" t="str">
+        <x:v>Ghi khi Sap item đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I55" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-58/63</x:v>
+      </x:c>
+      <x:c r="J55" s="18" t="str">
+        <x:v>Không nhận từ Chop Stump trong gói giấy; nguồn khác/công dụng để sau</x:v>
+      </x:c>
+      <x:c r="K55" s="18" t="str">
+        <x:v>Decision 09 · CG-58/63; Forest content batch 01; Stardew Wiki Trees/Mahogany Tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="62" customHeight="1">
+      <x:c r="A56" s="19" t="str">
+        <x:v>Apricot Tree</x:v>
+      </x:c>
+      <x:c r="B56" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C56" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D56" s="18" t="str">
+        <x:v>Plant Apricot Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E56" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F56" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Apricot; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G56" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Có quả / Đã hái 0/3; hồi sau 3 Spring Sleep</x:v>
+      </x:c>
+      <x:c r="H56" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I56" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J56" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K56" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="62" customHeight="1">
+      <x:c r="A57" s="19" t="str">
+        <x:v>Cherry Tree</x:v>
+      </x:c>
+      <x:c r="B57" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C57" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D57" s="18" t="str">
+        <x:v>Plant Cherry Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E57" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F57" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Cherry; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G57" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Có quả / Đã hái 0/3; hồi sau 3 Spring Sleep</x:v>
+      </x:c>
+      <x:c r="H57" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I57" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J57" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K57" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="62" customHeight="1">
+      <x:c r="A58" s="19" t="str">
+        <x:v>Apricot Sapling</x:v>
+      </x:c>
+      <x:c r="B58" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C58" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Apricot Tree</x:v>
+      </x:c>
+      <x:c r="D58" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E58" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F58" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Apricot Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G58" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H58" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I58" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J58" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K58" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="62" customHeight="1">
+      <x:c r="A59" s="19" t="str">
+        <x:v>Cherry Sapling</x:v>
+      </x:c>
+      <x:c r="B59" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C59" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Cherry Tree</x:v>
+      </x:c>
+      <x:c r="D59" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E59" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F59" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Cherry Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G59" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H59" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I59" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J59" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K59" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="62" customHeight="1">
+      <x:c r="A60" s="19" t="str">
+        <x:v>Apricot</x:v>
+      </x:c>
+      <x:c r="B60" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C60" s="18" t="str">
+        <x:v>Item sau Hand Harvest Apricot Tree</x:v>
+      </x:c>
+      <x:c r="D60" s="18" t="str">
+        <x:v>Mature Apricot Tree Có quả trong Spring</x:v>
+      </x:c>
+      <x:c r="E60" s="18" t="str">
+        <x:v>Hand → Apricot Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F60" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Apricot; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G60" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H60" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I60" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J60" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K60" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="62" customHeight="1">
+      <x:c r="A61" s="19" t="str">
+        <x:v>Cherry</x:v>
+      </x:c>
+      <x:c r="B61" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C61" s="18" t="str">
+        <x:v>Item sau Hand Harvest Cherry Tree</x:v>
+      </x:c>
+      <x:c r="D61" s="18" t="str">
+        <x:v>Mature Cherry Tree Có quả trong Spring</x:v>
+      </x:c>
+      <x:c r="E61" s="18" t="str">
+        <x:v>Hand → Cherry Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F61" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Cherry; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G61" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H61" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I61" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-59</x:v>
+      </x:c>
+      <x:c r="J61" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K61" s="18" t="str">
+        <x:v>Decision 09 · CG-59; Fruit Tree content batch 01; Stardew Wiki Fruit Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="62" customHeight="1">
+      <x:c r="A62" s="19" t="str">
+        <x:v>Orange Tree</x:v>
+      </x:c>
+      <x:c r="B62" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C62" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D62" s="18" t="str">
+        <x:v>Plant Orange Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E62" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F62" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Orange; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G62" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Summer Có quả / Đã hái 0/3; hồi sau 3 Summer Sleep</x:v>
+      </x:c>
+      <x:c r="H62" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I62" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J62" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K62" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Orange Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="62" customHeight="1">
+      <x:c r="A63" s="19" t="str">
+        <x:v>Peach Tree</x:v>
+      </x:c>
+      <x:c r="B63" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C63" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D63" s="18" t="str">
+        <x:v>Plant Peach Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E63" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F63" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Peach; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G63" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Summer Có quả / Đã hái 0/3; hồi sau 3 Summer Sleep</x:v>
+      </x:c>
+      <x:c r="H63" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I63" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J63" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K63" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Peach Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="62" customHeight="1">
+      <x:c r="A64" s="19" t="str">
+        <x:v>Orange Sapling</x:v>
+      </x:c>
+      <x:c r="B64" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C64" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Orange Tree</x:v>
+      </x:c>
+      <x:c r="D64" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E64" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F64" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Orange Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G64" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H64" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I64" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J64" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K64" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Orange Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="62" customHeight="1">
+      <x:c r="A65" s="19" t="str">
+        <x:v>Peach Sapling</x:v>
+      </x:c>
+      <x:c r="B65" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C65" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Peach Tree</x:v>
+      </x:c>
+      <x:c r="D65" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E65" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F65" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Peach Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G65" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H65" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I65" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J65" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K65" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Peach Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="62" customHeight="1">
+      <x:c r="A66" s="19" t="str">
+        <x:v>Orange</x:v>
+      </x:c>
+      <x:c r="B66" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C66" s="18" t="str">
+        <x:v>Item sau Hand Harvest Orange Tree</x:v>
+      </x:c>
+      <x:c r="D66" s="18" t="str">
+        <x:v>Mature Orange Tree Có quả trong Summer</x:v>
+      </x:c>
+      <x:c r="E66" s="18" t="str">
+        <x:v>Hand → Orange Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F66" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Orange; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G66" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H66" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I66" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J66" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K66" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Orange Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="62" customHeight="1">
+      <x:c r="A67" s="19" t="str">
+        <x:v>Peach</x:v>
+      </x:c>
+      <x:c r="B67" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C67" s="18" t="str">
+        <x:v>Item sau Hand Harvest Peach Tree</x:v>
+      </x:c>
+      <x:c r="D67" s="18" t="str">
+        <x:v>Mature Peach Tree Có quả trong Summer</x:v>
+      </x:c>
+      <x:c r="E67" s="18" t="str">
+        <x:v>Hand → Peach Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F67" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Peach; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G67" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H67" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I67" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-60</x:v>
+      </x:c>
+      <x:c r="J67" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K67" s="18" t="str">
+        <x:v>Decision 09 · CG-60; Fruit Tree content batch 01; Stardew Wiki Peach Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="62" customHeight="1">
+      <x:c r="A68" s="19" t="str">
+        <x:v>Apple Tree</x:v>
+      </x:c>
+      <x:c r="B68" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C68" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D68" s="18" t="str">
+        <x:v>Plant Apple Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E68" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F68" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Apple; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G68" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Fall Có quả / Đã hái 0/3; hồi sau 3 Fall Sleep</x:v>
+      </x:c>
+      <x:c r="H68" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I68" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J68" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K68" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Apple Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="62" customHeight="1">
+      <x:c r="A69" s="19" t="str">
+        <x:v>Pomegranate Tree</x:v>
+      </x:c>
+      <x:c r="B69" s="18" t="str">
+        <x:v>Vegetation · cây ăn quả bám đất</x:v>
+      </x:c>
+      <x:c r="C69" s="18" t="str">
+        <x:v>Tableau Home → Field; chiếm 1/8 vị trí</x:v>
+      </x:c>
+      <x:c r="D69" s="18" t="str">
+        <x:v>Plant Pomegranate Sapling trên Empty/Tilled Soil; Young 0/6</x:v>
+      </x:c>
+      <x:c r="E69" s="18" t="str">
+        <x:v>Sapling → Soil; Hand → cây Có quả; Axe → cây</x:v>
+      </x:c>
+      <x:c r="F69" s="18" t="str">
+        <x:v>Plant 1 AP; 6 Sleep để Mature; Harvest 1 AP cho 1 Pomegranate; Chop 1 AP trả sapling, Mature thêm 2 Wood</x:v>
+      </x:c>
+      <x:c r="G69" s="18" t="str">
+        <x:v>Young 0/6 → Mature; Fall Có quả / Đã hái 0/3; hồi sau 3 Fall Sleep</x:v>
+      </x:c>
+      <x:c r="H69" s="18" t="str">
+        <x:v>Ghi khi chính lá cây hiện sau Plant</x:v>
+      </x:c>
+      <x:c r="I69" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J69" s="18" t="str">
+        <x:v>Chưa có giá, art; không tưới, không Stump</x:v>
+      </x:c>
+      <x:c r="K69" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Pomegranate Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="62" customHeight="1">
+      <x:c r="A70" s="19" t="str">
+        <x:v>Apple Sapling</x:v>
+      </x:c>
+      <x:c r="B70" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C70" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Apple Tree</x:v>
+      </x:c>
+      <x:c r="D70" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E70" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F70" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Apple Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G70" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H70" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I70" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J70" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K70" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Apple Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="62" customHeight="1">
+      <x:c r="A71" s="19" t="str">
+        <x:v>Pomegranate Sapling</x:v>
+      </x:c>
+      <x:c r="B71" s="18" t="str">
+        <x:v>Item / Seed · Sapling</x:v>
+      </x:c>
+      <x:c r="C71" s="18" t="str">
+        <x:v>Item từ đầu V0; trở lại Item sau Chop Pomegranate Tree</x:v>
+      </x:c>
+      <x:c r="D71" s="18" t="str">
+        <x:v>Có 1 từ đầu; không có shop V0</x:v>
+      </x:c>
+      <x:c r="E71" s="18" t="str">
+        <x:v>Chọn trong Item → Empty/Tilled Soil ở Field</x:v>
+      </x:c>
+      <x:c r="F71" s="18" t="str">
+        <x:v>Plant 1 AP tiêu 1 sapling, thay Soil bằng Pomegranate Tree Young 0/6; Chop trả lại đúng sapling</x:v>
+      </x:c>
+      <x:c r="G71" s="18" t="str">
+        <x:v>Item giữ qua Sleep/Season; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H71" s="18" t="str">
+        <x:v>Ghi khi item đầu game hiện</x:v>
+      </x:c>
+      <x:c r="I71" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J71" s="18" t="str">
+        <x:v>Giá/nguồn bổ sung để sau</x:v>
+      </x:c>
+      <x:c r="K71" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Pomegranate Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="62" customHeight="1">
+      <x:c r="A72" s="19" t="str">
+        <x:v>Apple</x:v>
+      </x:c>
+      <x:c r="B72" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C72" s="18" t="str">
+        <x:v>Item sau Hand Harvest Apple Tree</x:v>
+      </x:c>
+      <x:c r="D72" s="18" t="str">
+        <x:v>Mature Apple Tree Có quả trong Fall</x:v>
+      </x:c>
+      <x:c r="E72" s="18" t="str">
+        <x:v>Hand → Apple Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F72" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Apple; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G72" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H72" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I72" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J72" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K72" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Apple Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="62" customHeight="1">
+      <x:c r="A73" s="19" t="str">
+        <x:v>Pomegranate</x:v>
+      </x:c>
+      <x:c r="B73" s="18" t="str">
+        <x:v>Item · Crop · fruit</x:v>
+      </x:c>
+      <x:c r="C73" s="18" t="str">
+        <x:v>Item sau Hand Harvest Pomegranate Tree</x:v>
+      </x:c>
+      <x:c r="D73" s="18" t="str">
+        <x:v>Mature Pomegranate Tree Có quả trong Fall</x:v>
+      </x:c>
+      <x:c r="E73" s="18" t="str">
+        <x:v>Hand → Pomegranate Tree Có quả</x:v>
+      </x:c>
+      <x:c r="F73" s="18" t="str">
+        <x:v>Harvest 1 AP cho 1 Pomegranate; cây ở lại và Đã hái 0/3</x:v>
+      </x:c>
+      <x:c r="G73" s="18" t="str">
+        <x:v>Một identity Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="H73" s="18" t="str">
+        <x:v>Ghi khi item quả đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I73" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-61</x:v>
+      </x:c>
+      <x:c r="J73" s="18" t="str">
+        <x:v>Giá, recipe, Gift và Processing để sau</x:v>
+      </x:c>
+      <x:c r="K73" s="18" t="str">
+        <x:v>Decision 09 · CG-61; Fruit Tree content batch 01; Stardew Wiki Pomegranate Sapling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="62" customHeight="1">
+      <x:c r="A74" s="19" t="str">
+        <x:v>Mahogany Tree</x:v>
+      </x:c>
+      <x:c r="B74" s="18" t="str">
+        <x:v>Vegetation · cây bám đất</x:v>
+      </x:c>
+      <x:c r="C74" s="18" t="str">
+        <x:v>Tableau Forest</x:v>
+      </x:c>
+      <x:c r="D74" s="18" t="str">
+        <x:v>Một lá Mature từ đầu; đã dọn trở lại Mature đầu Season kế</x:v>
+      </x:c>
+      <x:c r="E74" s="18" t="str">
+        <x:v>Axe → Mahogany Tree Mature hoặc Stump</x:v>
+      </x:c>
+      <x:c r="F74" s="18" t="str">
+        <x:v>Mature Chop 1 AP: 2 Hardwood + 1 Sap, thành Stump; Chop Stump 1 AP: +1 Wood, rời Forest</x:v>
+      </x:c>
+      <x:c r="G74" s="18" t="str">
+        <x:v>Mature / Stump / đã dọn; Sleep giữ state; Stump chưa dọn chặn hồi</x:v>
+      </x:c>
+      <x:c r="H74" s="18" t="str">
+        <x:v>Ghi khi lá cây lần đầu hiện ở Forest; Stump không có entry riêng</x:v>
+      </x:c>
+      <x:c r="I74" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể V0 · CG-63</x:v>
+      </x:c>
+      <x:c r="J74" s="18" t="str">
+        <x:v>Forest sẵn từ đầu là chuyển thể; Mahogany Seed, Tapper và sink Hardwood để sau</x:v>
+      </x:c>
+      <x:c r="K74" s="18" t="str">
+        <x:v>Decision 09 · CG-63; Forest content batch 01; Stardew Wiki Mahogany Tree/Trees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="62" customHeight="1">
+      <x:c r="A75" s="19" t="str">
+        <x:v>Hardwood</x:v>
+      </x:c>
+      <x:c r="B75" s="18" t="str">
+        <x:v>Item / material</x:v>
+      </x:c>
+      <x:c r="C75" s="18" t="str">
+        <x:v>Item sau Chop Mahogany Tree Mature ở Forest</x:v>
+      </x:c>
+      <x:c r="D75" s="18" t="str">
+        <x:v>Chop Mahogany Mature cho 2; Stump cho Wood</x:v>
+      </x:c>
+      <x:c r="E75" s="18" t="str">
+        <x:v>Output vào Item; giữ qua Sleep/Season</x:v>
+      </x:c>
+      <x:c r="F75" s="18" t="str">
+        <x:v>Chưa có recipe, giá bán, Bin hoặc Gift V0</x:v>
+      </x:c>
+      <x:c r="G75" s="18" t="str">
+        <x:v>Một identity Item riêng với Wood; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H75" s="18" t="str">
+        <x:v>Ghi khi Hardwood item đầu tiên hiện</x:v>
+      </x:c>
+      <x:c r="I75" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể output V0 · CG-63</x:v>
+      </x:c>
+      <x:c r="J75" s="18" t="str">
+        <x:v>Nguồn khác, giá và công dụng xử lý ở giai đoạn nội dung sau</x:v>
+      </x:c>
+      <x:c r="K75" s="18" t="str">
+        <x:v>Decision 09 · CG-63; Forest content batch 01; Stardew Wiki Hardwood/Mahogany Tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="62" customHeight="1">
+      <x:c r="A76" s="19" t="str">
+        <x:v>Chub</x:v>
+      </x:c>
+      <x:c r="B76" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C76" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D76" s="18" t="str">
+        <x:v>Cast thành công; Chub đủ điều kiện mọi Season</x:v>
+      </x:c>
+      <x:c r="E76" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F76" s="18" t="str">
+        <x:v>Nhận đúng 1 Chub nếu rút trúng từ tập Fish đủ Season; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G76" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H76" s="18" t="str">
+        <x:v>Ghi khi Chub item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I76" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể nội dung · CG-64</x:v>
+      </x:c>
+      <x:c r="J76" s="18" t="str">
+        <x:v>Giá bán, art và runtime còn mở; không gắn với spot/odds cụ thể</x:v>
+      </x:c>
+      <x:c r="K76" s="18" t="str">
+        <x:v>Decision 09 · CG-64; Fishing contract 01; River Fish batch 04; Stardew Wiki Chub</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="62" customHeight="1">
+      <x:c r="A77" s="19" t="str">
+        <x:v>Smallmouth Bass</x:v>
+      </x:c>
+      <x:c r="B77" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C77" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D77" s="18" t="str">
+        <x:v>Cast thành công trong Spring/Fall; rút trúng Smallmouth Bass</x:v>
+      </x:c>
+      <x:c r="E77" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F77" s="18" t="str">
+        <x:v>Nhận đúng 1 Smallmouth Bass nếu rút trúng từ tập Fish đủ Season; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G77" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H77" s="18" t="str">
+        <x:v>Ghi khi Smallmouth Bass item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I77" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể nội dung · CG-64</x:v>
+      </x:c>
+      <x:c r="J77" s="18" t="str">
+        <x:v>Không có trong pool Summer/Winter; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K77" s="18" t="str">
+        <x:v>Decision 09 · CG-64; Fishing contract 01; River Fish batch 04; Stardew Wiki Smallmouth Bass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="62" customHeight="1">
+      <x:c r="A78" s="19" t="str">
+        <x:v>Pike</x:v>
+      </x:c>
+      <x:c r="B78" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C78" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D78" s="18" t="str">
+        <x:v>Cast thành công trong Summer/Winter; rút trúng Pike</x:v>
+      </x:c>
+      <x:c r="E78" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F78" s="18" t="str">
+        <x:v>Nhận đúng 1 Pike nếu rút trúng từ tập Fish đủ Season; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G78" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H78" s="18" t="str">
+        <x:v>Ghi khi Pike item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I78" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể nội dung · CG-64</x:v>
+      </x:c>
+      <x:c r="J78" s="18" t="str">
+        <x:v>Không có trong pool Spring/Fall; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K78" s="18" t="str">
+        <x:v>Decision 09 · CG-64; Fishing contract 01; River Fish batch 04; Stardew Wiki Pike</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="62" customHeight="1">
+      <x:c r="A79" s="19" t="str">
+        <x:v>Perch</x:v>
+      </x:c>
+      <x:c r="B79" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C79" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D79" s="18" t="str">
+        <x:v>Cast thành công trong Winter; rút trúng Perch</x:v>
+      </x:c>
+      <x:c r="E79" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F79" s="18" t="str">
+        <x:v>Nhận đúng 1 Perch nếu rút trúng từ tập Fish đủ Season; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G79" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H79" s="18" t="str">
+        <x:v>Ghi khi Perch item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I79" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể nội dung · CG-64</x:v>
+      </x:c>
+      <x:c r="J79" s="18" t="str">
+        <x:v>Chỉ trong pool Winter; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K79" s="18" t="str">
+        <x:v>Decision 09 · CG-64; Fishing contract 01; River Fish batch 04; Stardew Wiki Perch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="62" customHeight="1">
+      <x:c r="A80" s="19" t="str">
+        <x:v>Shad</x:v>
+      </x:c>
+      <x:c r="B80" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C80" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D80" s="18" t="str">
+        <x:v>Cast thành công, Today Weather Rain trong Spring/Summer/Fall, mọi pha; rút trúng Shad</x:v>
+      </x:c>
+      <x:c r="E80" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F80" s="18" t="str">
+        <x:v>Nhận đúng 1 Shad nếu rút trúng từ tập Fish đủ Season/Weather; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G80" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H80" s="18" t="str">
+        <x:v>Ghi khi Shad item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I80" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể Rain/giờ · CG-65</x:v>
+      </x:c>
+      <x:c r="J80" s="18" t="str">
+        <x:v>Khung 9am–2am nguồn được nén thành ngày giấy; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K80" s="18" t="str">
+        <x:v>Decision 09 · CG-65; Fishing contract 01; River Fish batch 04; Stardew Wiki Shad</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="62" customHeight="1">
+      <x:c r="A81" s="19" t="str">
+        <x:v>Catfish</x:v>
+      </x:c>
+      <x:c r="B81" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C81" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D81" s="18" t="str">
+        <x:v>Cast thành công, Today Weather Rain trong Spring/Fall, mọi pha; rút trúng Catfish</x:v>
+      </x:c>
+      <x:c r="E81" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F81" s="18" t="str">
+        <x:v>Nhận đúng 1 Catfish nếu rút trúng từ tập Fish đủ Season/Weather; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G81" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H81" s="18" t="str">
+        <x:v>Ghi khi Catfish item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I81" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể Rain/giờ · CG-65</x:v>
+      </x:c>
+      <x:c r="J81" s="18" t="str">
+        <x:v>Khung 6am–12am nguồn được nén; không nhập Secret Woods/Rain Totem; giá, art/runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K81" s="18" t="str">
+        <x:v>Decision 09 · CG-65; Fishing contract 01; River Fish batch 04; Stardew Wiki Catfish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="62" customHeight="1">
+      <x:c r="A82" s="19" t="str">
+        <x:v>Walleye</x:v>
+      </x:c>
+      <x:c r="B82" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C82" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D82" s="18" t="str">
+        <x:v>Cast thành công trong Fall, Today Weather Rain, pha Noon/Afternoon/Night; rút trúng Walleye</x:v>
+      </x:c>
+      <x:c r="E82" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F82" s="18" t="str">
+        <x:v>Nhận đúng 1 Walleye nếu rút trúng từ tập Fish đủ Season/Weather/pha; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G82" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H82" s="18" t="str">
+        <x:v>Ghi khi Walleye item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I82" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể pha · CG-66/67</x:v>
+      </x:c>
+      <x:c r="J82" s="18" t="str">
+        <x:v>Winter Rain Totem chưa có V0; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K82" s="18" t="str">
+        <x:v>Decision 09 · CG-66/67; Fishing contract 01; River Fish batch 04; Stardew Wiki Walleye</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="62" customHeight="1">
+      <x:c r="A83" s="19" t="str">
+        <x:v>Sunfish</x:v>
+      </x:c>
+      <x:c r="B83" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C83" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D83" s="18" t="str">
+        <x:v>Cast thành công trong Spring/Summer, Today Weather Sunny, pha Morning/Noon/Afternoon; rút trúng Sunfish</x:v>
+      </x:c>
+      <x:c r="E83" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F83" s="18" t="str">
+        <x:v>Nhận đúng 1 Sunfish nếu rút trúng từ tập Fish đủ Season/Weather/pha; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G83" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H83" s="18" t="str">
+        <x:v>Ghi khi Sunfish item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I83" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể Sunny/pha · CG-67</x:v>
+      </x:c>
+      <x:c r="J83" s="18" t="str">
+        <x:v>Wind trong nguồn để sau; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K83" s="18" t="str">
+        <x:v>Decision 09 · CG-67; Fishing contract 01; River Fish batch 04; Stardew Wiki Sunfish</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="62" customHeight="1">
+      <x:c r="A84" s="19" t="str">
+        <x:v>Rainbow Trout</x:v>
+      </x:c>
+      <x:c r="B84" s="18" t="str">
+        <x:v>Item · Fish</x:v>
+      </x:c>
+      <x:c r="C84" s="18" t="str">
+        <x:v>River → Item</x:v>
+      </x:c>
+      <x:c r="D84" s="18" t="str">
+        <x:v>Cast thành công trong Summer, Today Weather Sunny, pha Morning/Noon/Afternoon; rút trúng Rainbow Trout</x:v>
+      </x:c>
+      <x:c r="E84" s="18" t="str">
+        <x:v>Fish vào Item; có thể gửi Shipping Bin</x:v>
+      </x:c>
+      <x:c r="F84" s="18" t="str">
+        <x:v>Nhận đúng 1 Rainbow Trout nếu rút trúng từ tập Fish đủ Season/Weather/pha; Gold qua Bin đến cuối ngày</x:v>
+      </x:c>
+      <x:c r="G84" s="18" t="str">
+        <x:v>Fresh; số lượng trong Item</x:v>
+      </x:c>
+      <x:c r="H84" s="18" t="str">
+        <x:v>Ghi khi Rainbow Trout item lần đầu hiện; thấy Spot chưa ghi Fish</x:v>
+      </x:c>
+      <x:c r="I84" s="18" t="str">
+        <x:v>Lựa chọn chuyển thể Sunny/pha · CG-67</x:v>
+      </x:c>
+      <x:c r="J84" s="18" t="str">
+        <x:v>Trout Derby trong nguồn để sau; giá, art và runtime còn mở</x:v>
+      </x:c>
+      <x:c r="K84" s="18" t="str">
+        <x:v>Decision 09 · CG-67; Fishing contract 01; River Fish batch 04; Stardew Wiki Rainbow Trout</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="62" customHeight="1">
+      <x:c r="A85" s="24" t="str">
+        <x:v>Farm Pond</x:v>
+      </x:c>
+      <x:c r="B85" s="25" t="str">
+        <x:v>Source card</x:v>
+      </x:c>
+      <x:c r="C85" s="25" t="str">
+        <x:v>Home tableau; ngoài sức chứa đất Field</x:v>
+      </x:c>
+      <x:c r="D85" s="25" t="str">
+        <x:v>Có sẵn khi mở Home; lá hiện trực tiếp cạnh Field/Farmhouse/Bin</x:v>
+      </x:c>
+      <x:c r="E85" s="25" t="str">
+        <x:v>Watering Can → Múc nước; không là River/Fishing Spot</x:v>
+      </x:c>
+      <x:c r="F85" s="25" t="str">
+        <x:v>Nạp đầy Can 0 AP; Pond không spent; Water trên crop vẫn trả 1 AP và dùng một lượng nước</x:v>
+      </x:c>
+      <x:c r="G85" s="25" t="str">
+        <x:v>Nguồn nước thường trực; lượng nước hiện trên Can, không trên Pond</x:v>
+      </x:c>
+      <x:c r="H85" s="25" t="str">
+        <x:v>Ghi Farm Pond khi lá lần đầu hiện ở Home</x:v>
+      </x:c>
+      <x:c r="I85" s="25" t="str">
+        <x:v>Owner yêu cầu lá nguồn Home · CG-69; action là lựa chọn chuyển thể</x:v>
+      </x:c>
+      <x:c r="J85" s="25" t="str">
+        <x:v>40 lượng trong prototype là fixture từ Watering Can thường Stardew; art/cân bằng cuối còn mở</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>Decision 09 · CG-18/22–24/64–67; Fishing contract 01; River Fish batch 04</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf8386cff3f4757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6016c9f90f934e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>